<commit_message>
Correct the cost framing and add the pricing model tab
The 1,851 PLN per client was a fully-loaded figure presented as cash: it
included the whole platform cost divided by one client (770 PLN) and notional
founder time (300 PLN), neither of which is money leaving the account. The
marginal cash cost is 781 PLN at the assumed volumes.

Adds a Model cenowy tab with three volume scenarios. Cash cost per client runs
196 PLN at low volume to 1,482 PLN at high, a 7.6x spread, which is the
argument that a seat cap alone cannot bound cost. Also sets out the comparison
frames: a retainer competes with an SDR at 8,500-11,000 PLN, while per-seat
pricing competes with Pipedrive and lands 4x above the top of the Polish market.

Margins come off the deck until the volumes are measured on the four testing
companies.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsD4eYJwPAt1SuH7uuTPjd
</commit_message>
<xml_diff>
--- a/analysis/model-valenos.xlsx
+++ b/analysis/model-valenos.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Plan 12 miesiecy" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Kohorta founding" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Wykorzystanie srodkow" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Model cenowy" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1251,6 +1252,141 @@
       <c r="D69" s="2" t="inlineStr">
         <is>
           <t>Zalozenie</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Scenariusze wolumenu agenta na klienta (miesiecznie)</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Pozycja</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Niski</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>Sredni</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Wysoki</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Firmy przeskanowane</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="C73" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Firmy wzbogacone</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C74" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Kontakty wzbogacone</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C75" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Maile wyslane</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="C76" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Akcje agenta CRM</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Dane na klienta (PLN)</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="C78" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Scenariusze sa ZALOZENIEM. Zmierz je na czterech firmach testujacych i wpisz prawdziwe liczby.</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1277,7 +1413,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Koszt obslugi jednego klienta miesiecznie (PLN)</t>
+          <t>Koszt obslugi: gotowka a koszt pelny</t>
         </is>
       </c>
     </row>
@@ -1401,15 +1537,26 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Inferencja nie spada ze skala: ta sama kwota przy 1 i przy 50 klientach. To jedyny koszt, ktory zostaje.</t>
+          <t>UWAGA: wiersz Razem to koszt PELNY, czyli z infrastruktura platformy podzielona przez liczbe klientow i z wycenionym czasem zalozycieli.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Przy braku optymalizacji ekstrakcji tresci (0,60 USD za firme zamiast 0,15) inferencja rosnie ok. 2,4x - zmien B7 w Zalozeniach i zobacz skutek.</t>
-        </is>
+          <t>Gotowka wychodzaca to tylko inferencja plus dane. Przy jednym kliencie infrastruktura to cala platforma, a nie koszt tego klienta. Patrz zakladka Model cenowy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Koszt krancowy gotowkowy na klienta (sredni wolumen)</t>
+        </is>
+      </c>
+      <c r="B12" s="26">
+        <f>B4+B5</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3481,4 +3628,313 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model cenowy: co naprawde kosztuje obsluga klienta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tylko gotowka wychodzaca. Infrastruktura platformy i czas zalozycieli NIE sa kosztem na klienta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Skladnik</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Niski wolumen</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Sredni wolumen</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Wysoki wolumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Inferencja modelowa</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>('Zalozenia'!$B$6*'Zalozenia'!$B$73+'Zalozenia'!$B$7*'Zalozenia'!$B$74+'Zalozenia'!$B$8*'Zalozenia'!$B$75+'Zalozenia'!$B$9*'Zalozenia'!$B$76+'Zalozenia'!$B$10*'Zalozenia'!$B$77)*'Zalozenia'!$B$3</f>
+        <v/>
+      </c>
+      <c r="C5" s="16">
+        <f>('Zalozenia'!$B$6*'Zalozenia'!$C$73+'Zalozenia'!$B$7*'Zalozenia'!$C$74+'Zalozenia'!$B$8*'Zalozenia'!$C$75+'Zalozenia'!$B$9*'Zalozenia'!$C$76+'Zalozenia'!$B$10*'Zalozenia'!$C$77)*'Zalozenia'!$B$3</f>
+        <v/>
+      </c>
+      <c r="D5" s="16">
+        <f>('Zalozenia'!$B$6*'Zalozenia'!$D$73+'Zalozenia'!$B$7*'Zalozenia'!$D$74+'Zalozenia'!$B$8*'Zalozenia'!$D$75+'Zalozenia'!$B$9*'Zalozenia'!$D$76+'Zalozenia'!$B$10*'Zalozenia'!$D$77)*'Zalozenia'!$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dane: Apollo, wyszukiwarka, weryfikacja</t>
+        </is>
+      </c>
+      <c r="B6" s="16">
+        <f>'Zalozenia'!$B$78</f>
+        <v/>
+      </c>
+      <c r="C6" s="16">
+        <f>'Zalozenia'!$C$78</f>
+        <v/>
+      </c>
+      <c r="D6" s="16">
+        <f>'Zalozenia'!$D$78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Koszt krancowy gotowkowy na klienta</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="15">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Rozpietosc miedzy najlzejszym a najciezszym klientem</t>
+        </is>
+      </c>
+      <c r="B9" s="29">
+        <f>D7/B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Limit stanowisk NIE ogranicza tej rozpietosci. Ten sam klient moze miec 3 stanowiska przy kazdym z tych wolumenow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Koszt krancowy jako udzial ceny</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Cena abonamentu</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Niski</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Sredni</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Wysoki</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16">
+        <f>'Zalozenia'!$B$31</f>
+        <v/>
+      </c>
+      <c r="B15" s="17">
+        <f>B$7/$A15</f>
+        <v/>
+      </c>
+      <c r="C15" s="17">
+        <f>C$7/$A15</f>
+        <v/>
+      </c>
+      <c r="D15" s="17">
+        <f>D$7/$A15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16">
+        <f>'Zalozenia'!$B$32</f>
+        <v/>
+      </c>
+      <c r="B16" s="17">
+        <f>B$7/$A16</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>C$7/$A16</f>
+        <v/>
+      </c>
+      <c r="D16" s="17">
+        <f>D$7/$A16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Rama porownawcza dla kupujacego (PLN/mies., szacunki rynkowe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Alternatywa klienta</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Od</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Do</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Junior SDR, pelny koszt pracodawcy</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>8500</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Agencja outboundowa, retainer</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CRM rozliczany per stanowisko, 5 stanowisk</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>245</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>ValenOS przy cenie standard</t>
+        </is>
+      </c>
+      <c r="B25" s="26">
+        <f>'Zalozenia'!$B$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Przy wycenie per stanowisko, 5 stanowisk, wyszloby na stanowisko</t>
+        </is>
+      </c>
+      <c r="B26" s="16">
+        <f>'Zalozenia'!$B$32/5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Gorna granica polskiego rynku CRM za stanowisko</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ile razy powyzej rynku</t>
+        </is>
+      </c>
+      <c r="B28" s="29">
+        <f>B26/B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Wniosek: retainer ustawia porownanie z kosztem handlowca lub agencji, gdzie ValenOS wygrywa. Wycena per stanowisko ustawia porownanie z Pipedrive, gdzie przegrywa 4x.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>